<commit_message>
Archive hoveniers50_enriched.xlsx from ecoscrape: First 50 hoveniers enriched, deeper email regex scan added 15 more emails and 14 more phones
</commit_message>
<xml_diff>
--- a/projects/ecoscrape/spreadsheets/hoveniers50_enriched.xlsx
+++ b/projects/ecoscrape/spreadsheets/hoveniers50_enriched.xlsx
@@ -763,8 +763,16 @@
           <t>9468 BN</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>info@wijnholdstuinen.nl</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0623758480</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>https://www.wijnholdstuinen.nl/</t>
@@ -1119,8 +1127,16 @@
           <t>9404 GD</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>info@dewilgenhut.nl</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0624453187</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>http://www.dewilgenhut.nl/</t>
@@ -1387,8 +1403,16 @@
           <t>9407 PH</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>gsgroenservice@gmail.com</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0648600095</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>http://gsgroenservice.eu/</t>
@@ -1481,12 +1505,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>johanhaveman@home.nl</t>
+          <t>johanhaveman80@gmail.com</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0592404129</t>
+          <t>0655966556</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1581,7 +1605,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>info@hoveniersbedrijfmarcobakker.nl</t>
+          <t>info@marcobakkerdroomtuinen.nl</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1963,7 +1987,11 @@
           <t>9403 VS</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>info@mennegagroenvoorziening.nl</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
@@ -2055,8 +2083,16 @@
           <t>9407 JA</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>contact@pleziermetgroen.nl</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0652506530</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>https://www.pleziermetgroen.nl/</t>
@@ -2147,8 +2183,16 @@
           <t>9404 JJ</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>info@rsbestratingassen.nl</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0622995041</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>https://rsbestratingassen.nl/</t>
@@ -2240,7 +2284,11 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0643884015</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>https://www.thijms.nl/</t>
@@ -2595,7 +2643,11 @@
           <t>9403 SK</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>info@tuinservicehessels.nl</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
@@ -2687,8 +2739,16 @@
           <t>9408 JE</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>info@tuinservicescholing.nl</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>0620255441</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>https://tuinservicescholing.nl/</t>
@@ -2779,8 +2839,16 @@
           <t>9406 JR</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>info@tuinservicevanwattum.nl</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>0641505598</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>https://www.tuinservicevanwattum.nl/</t>
@@ -2871,8 +2939,16 @@
           <t>9402 JL</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>info@tuinservicevochteloo.nl</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0683578006</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>https://www.tuinservicevochteloo.nl/</t>
@@ -3151,8 +3227,16 @@
           <t>9412 AG</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>info@boerstuinklussen.nl</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>0613344165</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>https://boerstuinklussen.nl/</t>
@@ -3243,8 +3327,16 @@
           <t>9411 SE</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>info@dolmansdenboer.com</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>0478441004</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>https://www.dolmanslandscaping.com/</t>
@@ -3427,8 +3519,16 @@
           <t>9413 AC</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>info@korre.nl</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0622863027</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>https://www.korre.nl/</t>
@@ -3699,8 +3799,16 @@
           <t>9411 LT</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>info@vista-verde.nl</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>0619671804</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>https://www.vista-verde.nl/</t>
@@ -3971,8 +4079,16 @@
           <t>9528 PJ</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>info@brouwertuinwerken.nl</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>0611626896</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>https://www.brouwertuinwerken.nl/</t>
@@ -4713,12 +4829,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>jhm.timmer@curatio.nl</t>
+          <t>vragen@curatio.nl</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>+31524208005</t>
+          <t>0524552284</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">

</xml_diff>